<commit_message>
Oct 9 refresh: W9/W10 true-up from the Oct 9 MMC export, tracker W8–W10, W11–W16 plan on actual check-ins
- Recap of the first two new-cadence weeks against the Sep 22 plan (planned vs checked-in, off-plan book visits by tier, visit-days); ledger W9/W10 rows carry actual_status
- Tracker check-ins W8 (Sep 3 tiers), W9, W10 (Sep 22 tiers), visit-day basis
- Clocks reset to actual check-ins through Oct 9; cells unchanged; W11–W16 (Oct 12 → Nov 20) rebuilt with the Sep 22 composer; ledger, scheduled days, app (14 weeks), MMC import First Planned Week, three PL workbooks + dated 2026-10-09 copies
- Relationship workbook visit-days extended to Oct 9; parking-lot Oct 9 refresh section; plan doc v14 banner

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ei2NMkxuP1dquQsjedq4wC
</commit_message>
<xml_diff>
--- a/pm/b2b-relationship-opportunities-2026.xlsx
+++ b/pm/b2b-relationship-opportunities-2026.xlsx
@@ -490,7 +490,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Basis: Jan 1–Sep 25 B2B referrals mapped to MMC companies (b2b-spine-growth-2026.xlsx) × the spine book (tier / PL / route day) × the MMC contact roster × completed visits Mar 3–Sep 22. Referrer-side aggregates only; no patient data.</t>
+          <t>Basis: Jan 1–Sep 25 B2B referrals mapped to MMC companies (b2b-spine-growth-2026.xlsx) × the spine book (tier / PL / route day) × the MMC contact roster × completed visits Mar 3–Oct 9 (visit-days). Referrer-side aggregates only; no patient data.</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
     <row r="12" ht="48" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>7 · DORMANT (63): Tier 1/2 accounts with zero 2026 referrals of any kind — 13 had 3+ visit-days since Mar 3 with nothing back, 12 were never visited (33 Tier 1 · 30 Tier 2; 1 have referrals sitting on a sister MMC record — see_also). Re-qualify or move to Prospect; that is the visit capacity for buckets 2–5.</t>
+          <t>7 · DORMANT (63): Tier 1/2 accounts with zero 2026 referrals of any kind — 25 had 3+ visit-days Mar 3–Oct 9 with nothing back, 9 were never visited (33 Tier 1 · 30 Tier 2; 1 have referrals sitting on a sister MMC record — see_also). Re-qualify or move to Prospect; that is the visit capacity for buckets 2–5.</t>
         </is>
       </c>
     </row>
@@ -570,7 +570,7 @@
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>Pediatrics: 25 pediatric accounts are in the book as Tier 1/2 (61 visit-days since Mar 3, 6 spine all year; the type converts at 8%). They are the first candidates to move to Prospect when visit capacity is needed.</t>
+          <t>Pediatrics: 25 pediatric accounts are in the book as Tier 1/2 (68 visit-days since Mar 3, 6 spine all year; the type converts at 8%). They are the first candidates to move to Prospect when visit capacity is needed.</t>
         </is>
       </c>
     </row>
@@ -1074,10 +1074,10 @@
         </is>
       </c>
       <c r="C3" s="7" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D3" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E3" s="7" t="n">
         <v>0</v>
@@ -1095,10 +1095,10 @@
         </is>
       </c>
       <c r="C4" s="7" t="n">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="D4" s="7" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E4" s="7" t="n">
         <v>13</v>
@@ -1116,13 +1116,13 @@
         </is>
       </c>
       <c r="C5" s="7" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D5" s="7" t="n">
         <v>0</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="6">
@@ -1137,13 +1137,13 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D6" s="7" t="n">
         <v>12</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
     </row>
     <row r="7">
@@ -1158,10 +1158,10 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
@@ -1179,10 +1179,10 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>15</v>
@@ -1425,11 +1425,11 @@
         <v>2</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr">
@@ -1641,11 +1641,11 @@
         <v>2</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
@@ -1857,11 +1857,11 @@
         <v>2</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr">
@@ -2361,11 +2361,11 @@
         <v>4</v>
       </c>
       <c r="P16" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
@@ -2433,11 +2433,11 @@
         <v>6</v>
       </c>
       <c r="P17" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q17" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R17" s="7" t="inlineStr">
@@ -2577,11 +2577,11 @@
         <v>4</v>
       </c>
       <c r="P19" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
@@ -2721,11 +2721,11 @@
         <v>4</v>
       </c>
       <c r="P21" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr">
@@ -2793,11 +2793,11 @@
         <v>1</v>
       </c>
       <c r="P22" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
@@ -3009,11 +3009,11 @@
         <v>2</v>
       </c>
       <c r="P25" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
@@ -3225,11 +3225,11 @@
         <v>1</v>
       </c>
       <c r="P28" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
@@ -3369,11 +3369,11 @@
         <v>1</v>
       </c>
       <c r="P30" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q30" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R30" s="7" t="inlineStr">
@@ -3441,11 +3441,11 @@
         <v>14</v>
       </c>
       <c r="P31" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q31" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R31" s="7" t="inlineStr">
@@ -3585,11 +3585,11 @@
         <v>12</v>
       </c>
       <c r="P33" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q33" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R33" s="7" t="inlineStr">
@@ -3657,11 +3657,11 @@
         <v>6</v>
       </c>
       <c r="P34" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q34" s="7" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R34" s="7" t="inlineStr">
@@ -3801,11 +3801,11 @@
         <v>2</v>
       </c>
       <c r="P36" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q36" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R36" s="7" t="inlineStr">
@@ -4089,11 +4089,11 @@
         <v>4</v>
       </c>
       <c r="P40" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q40" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R40" s="7" t="inlineStr">
@@ -4161,11 +4161,11 @@
         <v>11</v>
       </c>
       <c r="P41" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q41" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R41" s="7" t="inlineStr">
@@ -4233,11 +4233,11 @@
         <v>8</v>
       </c>
       <c r="P42" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q42" s="7" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R42" s="7" t="inlineStr">
@@ -4305,11 +4305,11 @@
         <v>11</v>
       </c>
       <c r="P43" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q43" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R43" s="7" t="inlineStr">
@@ -4377,11 +4377,11 @@
         <v>6</v>
       </c>
       <c r="P44" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q44" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R44" s="7" t="inlineStr">
@@ -4449,11 +4449,11 @@
         <v>4</v>
       </c>
       <c r="P45" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q45" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="R45" s="7" t="inlineStr">
@@ -4521,11 +4521,11 @@
         <v>12</v>
       </c>
       <c r="P46" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q46" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R46" s="7" t="inlineStr">
@@ -4809,11 +4809,11 @@
         <v>11</v>
       </c>
       <c r="P50" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q50" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R50" s="7" t="inlineStr">
@@ -4881,11 +4881,11 @@
         <v>1</v>
       </c>
       <c r="P51" s="7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="Q51" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R51" s="7" t="inlineStr">
@@ -5165,11 +5165,11 @@
         <v>1</v>
       </c>
       <c r="P55" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q55" s="7" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R55" s="7" t="inlineStr">
@@ -5237,7 +5237,7 @@
         <v>7</v>
       </c>
       <c r="P56" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q56" s="7" t="inlineStr">
         <is>
@@ -5309,11 +5309,11 @@
         <v>2</v>
       </c>
       <c r="P57" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q57" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R57" s="7" t="inlineStr">
@@ -5381,11 +5381,11 @@
         <v>4</v>
       </c>
       <c r="P58" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q58" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R58" s="7" t="inlineStr">
@@ -5525,11 +5525,11 @@
         <v>4</v>
       </c>
       <c r="P60" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q60" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R60" s="7" t="inlineStr">
@@ -5669,11 +5669,11 @@
         <v>1</v>
       </c>
       <c r="P62" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q62" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R62" s="7" t="inlineStr">
@@ -5953,11 +5953,11 @@
         <v>20</v>
       </c>
       <c r="P66" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q66" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R66" s="7" t="inlineStr">
@@ -6025,11 +6025,11 @@
         <v>14</v>
       </c>
       <c r="P67" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q67" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R67" s="7" t="inlineStr">
@@ -6097,11 +6097,11 @@
         <v>9</v>
       </c>
       <c r="P68" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="Q68" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R68" s="7" t="inlineStr">
@@ -6169,11 +6169,11 @@
         <v>0</v>
       </c>
       <c r="P69" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q69" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R69" s="7" t="inlineStr">
@@ -6241,11 +6241,11 @@
         <v>2</v>
       </c>
       <c r="P70" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q70" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R70" s="7" t="inlineStr">
@@ -6313,11 +6313,11 @@
         <v>11</v>
       </c>
       <c r="P71" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q71" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R71" s="7" t="inlineStr">
@@ -6525,11 +6525,11 @@
         <v>0</v>
       </c>
       <c r="P74" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q74" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R74" s="7" t="inlineStr">
@@ -6813,11 +6813,11 @@
         <v>1</v>
       </c>
       <c r="P78" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q78" s="7" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R78" s="7" t="inlineStr">
@@ -7029,11 +7029,11 @@
         <v>26</v>
       </c>
       <c r="P81" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q81" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R81" s="7" t="inlineStr">
@@ -7173,11 +7173,11 @@
         <v>5</v>
       </c>
       <c r="P83" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q83" s="7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R83" s="7" t="inlineStr">
@@ -7385,11 +7385,11 @@
         <v>1</v>
       </c>
       <c r="P86" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q86" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="R86" s="7" t="inlineStr">
@@ -7457,11 +7457,11 @@
         <v>9</v>
       </c>
       <c r="P87" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q87" s="7" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="R87" s="7" t="inlineStr">
@@ -7529,11 +7529,11 @@
         <v>4</v>
       </c>
       <c r="P88" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q88" s="7" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R88" s="7" t="inlineStr">
@@ -7889,11 +7889,11 @@
         <v>3</v>
       </c>
       <c r="P93" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q93" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R93" s="7" t="inlineStr">
@@ -8033,11 +8033,11 @@
         <v>8</v>
       </c>
       <c r="P95" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q95" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R95" s="7" t="inlineStr">
@@ -8177,11 +8177,11 @@
         <v>2</v>
       </c>
       <c r="P97" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q97" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R97" s="7" t="inlineStr">
@@ -8321,11 +8321,11 @@
         <v>5</v>
       </c>
       <c r="P99" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q99" s="7" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R99" s="7" t="inlineStr">
@@ -8393,11 +8393,11 @@
         <v>2</v>
       </c>
       <c r="P100" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q100" s="7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R100" s="7" t="inlineStr">
@@ -8537,11 +8537,11 @@
         <v>3</v>
       </c>
       <c r="P102" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q102" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R102" s="7" t="inlineStr">
@@ -8753,11 +8753,11 @@
         <v>2</v>
       </c>
       <c r="P105" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q105" s="7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R105" s="7" t="inlineStr">
@@ -8897,11 +8897,11 @@
         <v>3</v>
       </c>
       <c r="P107" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q107" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R107" s="7" t="inlineStr">
@@ -9329,9 +9329,13 @@
         <v>5</v>
       </c>
       <c r="P113" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q113" s="7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Q113" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
       <c r="R113" s="7" t="inlineStr">
         <is>
           <t>2026-08-07</t>
@@ -9469,11 +9473,11 @@
         <v>2</v>
       </c>
       <c r="P115" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q115" s="7" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R115" s="7" t="inlineStr">
@@ -9541,11 +9545,11 @@
         <v>1</v>
       </c>
       <c r="P116" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q116" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R116" s="7" t="inlineStr">
@@ -9681,11 +9685,11 @@
         <v>7</v>
       </c>
       <c r="P118" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q118" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R118" s="7" t="inlineStr">
@@ -9969,11 +9973,11 @@
         <v>1</v>
       </c>
       <c r="P122" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q122" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R122" s="7" t="inlineStr">
@@ -10041,11 +10045,11 @@
         <v>1</v>
       </c>
       <c r="P123" s="7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="Q123" s="7" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R123" s="7" t="inlineStr">
@@ -10253,11 +10257,11 @@
         <v>9</v>
       </c>
       <c r="P126" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q126" s="7" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R126" s="7" t="inlineStr">
@@ -10325,11 +10329,11 @@
         <v>3</v>
       </c>
       <c r="P127" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q127" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R127" s="7" t="inlineStr">
@@ -10397,11 +10401,11 @@
         <v>1</v>
       </c>
       <c r="P128" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q128" s="7" t="inlineStr">
         <is>
-          <t>2026-05-06</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R128" s="7" t="inlineStr">
@@ -10469,11 +10473,11 @@
         <v>0</v>
       </c>
       <c r="P129" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q129" s="7" t="inlineStr">
         <is>
-          <t>2026-03-18</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R129" s="7" t="inlineStr">
@@ -10757,11 +10761,11 @@
         <v>1</v>
       </c>
       <c r="P133" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q133" s="7" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R133" s="7" t="inlineStr">
@@ -10829,11 +10833,11 @@
         <v>1</v>
       </c>
       <c r="P134" s="7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="Q134" s="7" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R134" s="7" t="inlineStr">
@@ -10901,11 +10905,11 @@
         <v>5</v>
       </c>
       <c r="P135" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q135" s="7" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="R135" s="7" t="inlineStr">
@@ -11181,11 +11185,11 @@
         <v>1</v>
       </c>
       <c r="P4" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R4" s="7" t="inlineStr">
@@ -11253,11 +11257,11 @@
         <v>0</v>
       </c>
       <c r="P5" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R5" s="7" t="inlineStr">
@@ -11325,11 +11329,11 @@
         <v>4</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
@@ -11397,11 +11401,11 @@
         <v>5</v>
       </c>
       <c r="P7" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
@@ -11469,11 +11473,11 @@
         <v>3</v>
       </c>
       <c r="P8" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr">
@@ -11685,11 +11689,11 @@
         <v>2</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q11" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R11" s="7" t="inlineStr">
@@ -11757,11 +11761,11 @@
         <v>2</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="R12" s="7" t="inlineStr">
@@ -11829,7 +11833,7 @@
         <v>0</v>
       </c>
       <c r="P13" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q13" s="7" t="inlineStr">
         <is>
@@ -11901,11 +11905,11 @@
         <v>8</v>
       </c>
       <c r="P14" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
@@ -12045,11 +12049,11 @@
         <v>3</v>
       </c>
       <c r="P16" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q16" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R16" s="7" t="inlineStr">
@@ -12189,11 +12193,11 @@
         <v>2</v>
       </c>
       <c r="P18" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q18" s="7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R18" s="7" t="inlineStr">
@@ -12333,11 +12337,11 @@
         <v>0</v>
       </c>
       <c r="P20" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="R20" s="7" t="inlineStr">
@@ -12405,11 +12409,11 @@
         <v>7</v>
       </c>
       <c r="P21" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R21" s="7" t="inlineStr">
@@ -12477,11 +12481,11 @@
         <v>6</v>
       </c>
       <c r="P22" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q22" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-10-02</t>
         </is>
       </c>
       <c r="R22" s="7" t="inlineStr">
@@ -12549,11 +12553,11 @@
         <v>2</v>
       </c>
       <c r="P23" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q23" s="7" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R23" s="7" t="inlineStr">
@@ -12621,11 +12625,11 @@
         <v>2</v>
       </c>
       <c r="P24" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q24" s="7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R24" s="7" t="inlineStr">
@@ -12693,11 +12697,11 @@
         <v>0</v>
       </c>
       <c r="P25" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q25" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R25" s="7" t="inlineStr">
@@ -12765,11 +12769,11 @@
         <v>3</v>
       </c>
       <c r="P26" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R26" s="7" t="inlineStr">
@@ -12909,11 +12913,11 @@
         <v>6</v>
       </c>
       <c r="P28" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q28" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R28" s="7" t="inlineStr">
@@ -13326,7 +13330,7 @@
         <v>4</v>
       </c>
       <c r="K4" s="7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L4" s="7" t="inlineStr">
         <is>
@@ -13374,7 +13378,7 @@
         <v>2</v>
       </c>
       <c r="K5" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
         <is>
@@ -13422,7 +13426,7 @@
         <v>1</v>
       </c>
       <c r="K6" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
         <is>
@@ -13518,7 +13522,7 @@
         <v>1</v>
       </c>
       <c r="K8" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
         <is>
@@ -13566,7 +13570,7 @@
         <v>1</v>
       </c>
       <c r="K9" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
         <is>
@@ -13710,7 +13714,7 @@
         <v>0</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
         <is>
@@ -13898,7 +13902,7 @@
         <v>0</v>
       </c>
       <c r="K16" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
@@ -13978,7 +13982,7 @@
         <v>0</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="L18" s="7" t="inlineStr"/>
     </row>
@@ -14018,7 +14022,7 @@
         <v>0</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L19" s="7" t="inlineStr"/>
     </row>
@@ -14873,11 +14877,11 @@
         <v>0</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr">
@@ -14945,11 +14949,11 @@
         <v>7</v>
       </c>
       <c r="P4" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="R4" s="7" t="inlineStr">
@@ -15089,11 +15093,11 @@
         <v>1</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
@@ -15297,11 +15301,11 @@
         <v>1</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr">
@@ -15513,11 +15517,11 @@
         <v>2</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
@@ -15585,11 +15589,11 @@
         <v>1</v>
       </c>
       <c r="P7" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R7" s="7" t="inlineStr">
@@ -15865,11 +15869,11 @@
         <v>2</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr">
@@ -16081,11 +16085,11 @@
         <v>6</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
@@ -16225,11 +16229,11 @@
         <v>3</v>
       </c>
       <c r="P8" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr"/>
@@ -16293,11 +16297,11 @@
         <v>3</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Q9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="R9" s="7" t="inlineStr">
@@ -16637,11 +16641,11 @@
         <v>3</v>
       </c>
       <c r="P14" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr"/>
@@ -16977,11 +16981,11 @@
         <v>3</v>
       </c>
       <c r="P3" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="R3" s="7" t="inlineStr">
@@ -17193,11 +17197,11 @@
         <v>9</v>
       </c>
       <c r="P6" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q6" s="7" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="R6" s="7" t="inlineStr">
@@ -17337,11 +17341,11 @@
         <v>3</v>
       </c>
       <c r="P8" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q8" s="7" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="R8" s="7" t="inlineStr">
@@ -17481,11 +17485,11 @@
         <v>12</v>
       </c>
       <c r="P10" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R10" s="7" t="inlineStr">
@@ -17625,11 +17629,11 @@
         <v>7</v>
       </c>
       <c r="P12" s="7" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="Q12" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-29</t>
         </is>
       </c>
       <c r="R12" s="7" t="inlineStr">
@@ -17769,11 +17773,11 @@
         <v>7</v>
       </c>
       <c r="P14" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-25</t>
         </is>
       </c>
       <c r="R14" s="7" t="inlineStr">
@@ -17841,11 +17845,11 @@
         <v>8</v>
       </c>
       <c r="P15" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q15" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R15" s="7" t="inlineStr">
@@ -18129,11 +18133,11 @@
         <v>3</v>
       </c>
       <c r="P19" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="Q19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="R19" s="7" t="inlineStr">
@@ -18201,11 +18205,11 @@
         <v>6</v>
       </c>
       <c r="P20" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q20" s="7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="R20" s="7" t="inlineStr">
@@ -18273,7 +18277,7 @@
         <v>7</v>
       </c>
       <c r="P21" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q21" s="7" t="inlineStr">
         <is>
@@ -19665,9 +19669,13 @@
         <v>1</v>
       </c>
       <c r="P23" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q23" s="7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="Q23" s="7" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
       <c r="R23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
@@ -19825,11 +19833,11 @@
         <v>3</v>
       </c>
       <c r="P26" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Q26" s="7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="R26" s="7" t="inlineStr"/>
@@ -22724,7 +22732,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Tier 1 / Tier 2 book accounts with no 2026 B2B referral of any service line. visits = visit-days (one PL at one practice on one date) Mar 3–Sep 22. Sorted by visit-days (most-visited first).</t>
+          <t>Tier 1 / Tier 2 book accounts with no 2026 B2B referral of any service line. visits = visit-days (one PL at one practice on one date) Mar 3–Oct 9. Sorted by visit-days (most-visited first).</t>
         </is>
       </c>
     </row>
@@ -22793,7 +22801,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>4 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
+          <t>5 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
@@ -22817,11 +22825,11 @@
         </is>
       </c>
       <c r="G3" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H3" s="7" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-09-28</t>
         </is>
       </c>
       <c r="I3" s="7" t="n">
@@ -22835,12 +22843,12 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>UNIVERSITY OF MICHIGAN LIVONIA HEALTH CENTER</t>
+          <t>Intensive Pulmonary &amp; Internal Medicine</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>4 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
+          <t>5 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -22855,7 +22863,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>J-A05</t>
+          <t>J-A06</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
@@ -22864,30 +22872,30 @@
         </is>
       </c>
       <c r="G4" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H4" s="7" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I4" s="7" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="K4" s="7" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="7" t="inlineStr">
         <is>
-          <t>Intensive Pulmonary &amp; Internal Medicine</t>
+          <t>Trinity Health IHA Medical Group, Hospital Medicine</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>4 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
+          <t>5 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C5" s="7" t="inlineStr">
@@ -22902,7 +22910,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>J-A06</t>
+          <t>J-A08</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
@@ -22911,30 +22919,30 @@
         </is>
       </c>
       <c r="G5" s="7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I5" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K5" s="7" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Trinity Health IHA Medical Group, Hospital Medicine</t>
+          <t>Wayne Primary Care and Walk In</t>
         </is>
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>4 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
+          <t>4 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits — NB: referrals from its clinicians sit on a sister record (see_also)</t>
         </is>
       </c>
       <c r="C6" s="7" t="inlineStr">
@@ -22954,7 +22962,7 @@
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Urgent care</t>
         </is>
       </c>
       <c r="G6" s="7" t="n">
@@ -22962,7 +22970,7 @@
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="I6" s="7" t="n">
@@ -22971,12 +22979,16 @@
       <c r="J6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="K6" s="7" t="inlineStr"/>
+      <c r="K6" s="7" t="inlineStr">
+        <is>
+          <t>Patel MD, Vijay (1) placed at GARDEN CITY FAMILY PHYSICIANS; PATEL MD, VIJAYKUMAR N (1) placed at GARDEN CITY FAMILY PHYSICIANS</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>Roger D Ajluni MD PC</t>
+          <t>UNIVERSITY OF MICHIGAN LIVONIA HEALTH CENTER</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
@@ -22991,12 +23003,12 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Jasmine</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
         <is>
-          <t>C-A14</t>
+          <t>J-A05</t>
         </is>
       </c>
       <c r="F7" s="7" t="inlineStr">
@@ -23009,21 +23021,21 @@
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="I7" s="7" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="K7" s="7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Schoenherr Internal Medicine</t>
+          <t>Roger D Ajluni MD PC</t>
         </is>
       </c>
       <c r="B8" s="7" t="inlineStr">
@@ -23038,12 +23050,12 @@
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>K-A12</t>
+          <t>C-A14</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -23056,21 +23068,21 @@
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="I8" s="7" t="n">
         <v>1</v>
       </c>
       <c r="J8" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K8" s="7" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="7" t="inlineStr">
         <is>
-          <t>Pioneer Medical Associates</t>
+          <t>MICHIGAN PREMIER INTERNISTS</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -23080,7 +23092,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -23090,7 +23102,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>K-A17</t>
+          <t>K-A18</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -23103,92 +23115,88 @@
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I9" s="7" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="K9" s="7" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Wayne Primary Care and Walk In</t>
+          <t>Clinton Preferred Pediatrics</t>
         </is>
       </c>
       <c r="B10" s="7" t="inlineStr">
         <is>
-          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits — NB: referrals from its clinicians sit on a sister record (see_also)</t>
+          <t>4 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Jasmine</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>J-A08</t>
+          <t>K-A08</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="G10" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="I10" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>Patel MD, Vijay (1) placed at GARDEN CITY FAMILY PHYSICIANS; PATEL MD, VIJAYKUMAR N (1) placed at GARDEN CITY FAMILY PHYSICIANS</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="K10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>Great Lakes Medicine</t>
+          <t>Schoenherr Internal Medicine</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
+          <t>4 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>C-A03</t>
+          <t>K-A12</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
@@ -23197,72 +23205,72 @@
         </is>
       </c>
       <c r="G11" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="I11" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K11" s="7" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>DEARBORN HEIGHTS MEDICAL CENTER</t>
+          <t>Pioneer Medical Associates</t>
         </is>
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
+          <t>4 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C12" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>C-A15</t>
+          <t>K-A17</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G12" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H12" s="7" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="I12" s="7" t="n">
-        <v>2</v>
+        <v>11</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="K12" s="7" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="7" t="inlineStr">
         <is>
-          <t>MICHIGAN PREMIER INTERNISTS</t>
+          <t>Osteopathic Health Care Associates</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
@@ -23272,17 +23280,17 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E13" s="7" t="inlineStr">
         <is>
-          <t>K-A18</t>
+          <t>C-A06</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -23295,21 +23303,21 @@
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I13" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="K13" s="7" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Clinton Preferred Pediatrics</t>
+          <t>Wayne state Internal Medicine</t>
         </is>
       </c>
       <c r="B14" s="7" t="inlineStr">
@@ -23324,17 +23332,17 @@
       </c>
       <c r="D14" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Jasmine</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
         <is>
-          <t>K-A08</t>
+          <t>J-A03</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G14" s="7" t="n">
@@ -23342,21 +23350,21 @@
       </c>
       <c r="H14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I14" s="7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K14" s="7" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>SG PEDIATRICS</t>
+          <t>Great Lakes Medicine</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
@@ -23366,22 +23374,22 @@
       </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>K-A20</t>
+          <t>C-A03</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G15" s="7" t="n">
@@ -23389,31 +23397,31 @@
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="I15" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K15" s="7" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Osteopathic Health Care Associates</t>
+          <t>JOEL WELLNESS CLINIC</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -23423,39 +23431,39 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>C-A06</t>
+          <t>C-A14</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="G16" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H16" s="7" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I16" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="K16" s="7" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>Wayne state Internal Medicine</t>
+          <t>DEARBORN HEIGHTS MEDICAL CENTER</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -23465,49 +23473,49 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>Jasmine</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
         <is>
-          <t>J-A03</t>
+          <t>C-A15</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="G17" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="I17" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K17" s="7" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>JOEL WELLNESS CLINIC</t>
+          <t>1st Choice Urgent Care- Rochester</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -23517,101 +23525,101 @@
       </c>
       <c r="E18" s="7" t="inlineStr">
         <is>
-          <t>C-A14</t>
+          <t>C-A04</t>
         </is>
       </c>
       <c r="F18" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>Urgent care</t>
         </is>
       </c>
       <c r="G18" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H18" s="7" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I18" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>1st Choice Urgent Care- Rochester</t>
+          <t>WESTERN WAYNE PHYSICIANS, PLC</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Jasmine</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
         <is>
-          <t>C-A04</t>
+          <t>J-A10</t>
         </is>
       </c>
       <c r="F19" s="7" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="G19" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I19" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K19" s="7" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>Dynamic Healthcare</t>
+          <t>Office of Lillman Dwarka MD</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>Jasmine</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
         <is>
-          <t>J-A03</t>
+          <t>K-A12</t>
         </is>
       </c>
       <c r="F20" s="7" t="inlineStr">
@@ -23620,30 +23628,30 @@
         </is>
       </c>
       <c r="G20" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H20" s="7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="I20" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K20" s="7" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>White Lake Family Medicine</t>
+          <t>MALI AND MALI PEDIATRICS - use this one</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -23658,39 +23666,39 @@
       </c>
       <c r="E21" s="7" t="inlineStr">
         <is>
-          <t>K-A07</t>
+          <t>K-A05</t>
         </is>
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="G21" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I21" s="7" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="J21" s="7" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="K21" s="7" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Office of Lillman Dwarka MD</t>
+          <t>Franklin Medical Consultants</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -23705,7 +23713,7 @@
       </c>
       <c r="E22" s="7" t="inlineStr">
         <is>
-          <t>K-A12</t>
+          <t>K-A18</t>
         </is>
       </c>
       <c r="F22" s="7" t="inlineStr">
@@ -23714,30 +23722,30 @@
         </is>
       </c>
       <c r="G22" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H22" s="7" t="inlineStr">
         <is>
-          <t>2026-04-29</t>
+          <t>2026-10-05</t>
         </is>
       </c>
       <c r="I22" s="7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="K22" s="7" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>MALI AND MALI PEDIATRICS - use this one</t>
+          <t>ASCENSION MACOMB OAKLAND HOSPITAL MOTOR CITY INTERNISTS</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -23752,39 +23760,39 @@
       </c>
       <c r="E23" s="7" t="inlineStr">
         <is>
-          <t>K-A05</t>
+          <t>K-A17</t>
         </is>
       </c>
       <c r="F23" s="7" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G23" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I23" s="7" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>15</v>
+        <v>3</v>
       </c>
       <c r="K23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>Middlebelt Medical Center</t>
+          <t>Trinity Medical Center</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -23799,7 +23807,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>K-A24</t>
+          <t>K-A13</t>
         </is>
       </c>
       <c r="F24" s="7" t="inlineStr">
@@ -23808,11 +23816,11 @@
         </is>
       </c>
       <c r="G24" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H24" s="7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-10-07</t>
         </is>
       </c>
       <c r="I24" s="7" t="n">
@@ -23826,17 +23834,17 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>Core Med  - White Lake</t>
+          <t>Care Choice LLC</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -23846,7 +23854,7 @@
       </c>
       <c r="E25" s="7" t="inlineStr">
         <is>
-          <t>K-A07</t>
+          <t>K-A11</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
@@ -23855,35 +23863,35 @@
         </is>
       </c>
       <c r="G25" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I25" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="K25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>Franklin Medical Consultants</t>
+          <t>Henry Ford Ascension St John Children's Center</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
@@ -23893,44 +23901,44 @@
       </c>
       <c r="E26" s="7" t="inlineStr">
         <is>
-          <t>K-A18</t>
+          <t>K-A05</t>
         </is>
       </c>
       <c r="F26" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="G26" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
-          <t>2026-05-27</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I26" s="7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="K26" s="7" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>NORTHWAY MEDICAL CENTER</t>
+          <t>SG PEDIATRICS</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>3 visit-days since Mar 3, nothing back — re-qualify, or move to Prospect to free visits</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
@@ -23940,34 +23948,34 @@
       </c>
       <c r="E27" s="7" t="inlineStr">
         <is>
-          <t>K-A25</t>
+          <t>K-A20</t>
         </is>
       </c>
       <c r="F27" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="G27" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="I27" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>ASCENSION MACOMB OAKLAND HOSPITAL MOTOR CITY INTERNISTS</t>
+          <t>Corewell East Area Family Practice - Roseville</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
@@ -23977,17 +23985,17 @@
       </c>
       <c r="C28" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>K-A17</t>
+          <t>C-A08</t>
         </is>
       </c>
       <c r="F28" s="7" t="inlineStr">
@@ -24000,21 +24008,21 @@
       </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
-          <t>2026-04-24</t>
+          <t>2026-10-06</t>
         </is>
       </c>
       <c r="I28" s="7" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K28" s="7" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Trinity Medical Center</t>
+          <t>Michigan primary care center/urgent care</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -24024,17 +24032,17 @@
       </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Jasmine</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>K-A13</t>
+          <t>J-A07</t>
         </is>
       </c>
       <c r="F29" s="7" t="inlineStr">
@@ -24047,7 +24055,7 @@
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-09-24</t>
         </is>
       </c>
       <c r="I29" s="7" t="n">
@@ -24061,7 +24069,7 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Care Choice LLC</t>
+          <t>Dynamic Healthcare</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
@@ -24076,12 +24084,12 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Jasmine</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>K-A11</t>
+          <t>J-A03</t>
         </is>
       </c>
       <c r="F30" s="7" t="inlineStr">
@@ -24094,7 +24102,7 @@
       </c>
       <c r="H30" s="7" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I30" s="7" t="n">
@@ -24108,7 +24116,7 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>Henry Ford Ascension St John Children's Center</t>
+          <t>White Lake Family Medicine</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -24118,7 +24126,7 @@
       </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -24128,12 +24136,12 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>K-A05</t>
+          <t>K-A07</t>
         </is>
       </c>
       <c r="F31" s="7" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G31" s="7" t="n">
@@ -24141,21 +24149,21 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>2026-06-10</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="I31" s="7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="J31" s="7" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="K31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>AMITY INTERNAL MEDICINE, PC - MDVIP</t>
+          <t>Middlebelt Medical Center</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
@@ -24165,7 +24173,7 @@
       </c>
       <c r="C32" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -24175,7 +24183,7 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>K-A15</t>
+          <t>K-A24</t>
         </is>
       </c>
       <c r="F32" s="7" t="inlineStr">
@@ -24188,7 +24196,7 @@
       </c>
       <c r="H32" s="7" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="I32" s="7" t="n">
@@ -24202,7 +24210,7 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>LIVONIA MEDICAL CLINIC</t>
+          <t>Core Med  - White Lake</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -24212,7 +24220,7 @@
       </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -24222,7 +24230,7 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>K-A24</t>
+          <t>K-A07</t>
         </is>
       </c>
       <c r="F33" s="7" t="inlineStr">
@@ -24235,21 +24243,21 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="I33" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J33" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K33" s="7" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>Maplecrest Medical Urgent Care</t>
+          <t>Macomb Neurology Associates</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
@@ -24259,7 +24267,7 @@
       </c>
       <c r="C34" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -24269,12 +24277,12 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>K-A13</t>
+          <t>K-A19</t>
         </is>
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Urgent care</t>
+          <t>Neurology</t>
         </is>
       </c>
       <c r="G34" s="7" t="n">
@@ -24282,7 +24290,7 @@
       </c>
       <c r="H34" s="7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I34" s="7" t="n">
@@ -24296,7 +24304,7 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>Port Huron Family Care</t>
+          <t>Oakland Medical Center</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -24306,7 +24314,7 @@
       </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -24316,7 +24324,7 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>K-A02</t>
+          <t>K-A10</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -24329,21 +24337,21 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I35" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J35" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K35" s="7" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>Shelby Pediatric Associates &amp; Child Lung Center</t>
+          <t>NORTHWAY MEDICAL CENTER</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
@@ -24353,7 +24361,7 @@
       </c>
       <c r="C36" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -24363,12 +24371,12 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>K-A06</t>
+          <t>K-A25</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G36" s="7" t="n">
@@ -24376,21 +24384,21 @@
       </c>
       <c r="H36" s="7" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="I36" s="7" t="n">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="J36" s="7" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="K36" s="7" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>Marshall Family Chiropractic</t>
+          <t>AMITY INTERNAL MEDICINE, PC - MDVIP</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
@@ -24410,12 +24418,12 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>K-A03</t>
+          <t>K-A15</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Chiropractic</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G37" s="7" t="n">
@@ -24423,21 +24431,21 @@
       </c>
       <c r="H37" s="7" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="I37" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J37" s="7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K37" s="7" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Imlay City Family Practice</t>
+          <t>LIVONIA MEDICAL CLINIC</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
@@ -24457,7 +24465,7 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>K-A01</t>
+          <t>K-A24</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
@@ -24470,88 +24478,88 @@
       </c>
       <c r="H38" s="7" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="I38" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K38" s="7" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>M-15 Family Medical Center</t>
+          <t>Maplecrest Medical Urgent Care</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>1 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>C-A02</t>
+          <t>K-A13</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Urgent care</t>
         </is>
       </c>
       <c r="G39" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="I39" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="K39" s="7" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>McLaren Oakland Internal Medicine - Clarkston</t>
+          <t>Port Huron Family Care</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>1 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>C-A02</t>
+          <t>K-A02</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
@@ -24560,11 +24568,11 @@
         </is>
       </c>
       <c r="G40" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H40" s="7" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="I40" s="7" t="n">
@@ -24578,12 +24586,12 @@
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>Corewell East Area Family Practice - Roseville</t>
+          <t>Shelby Pediatric Associates &amp; Child Lung Center</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>1 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -24593,49 +24601,49 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>C-A08</t>
+          <t>K-A06</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="G41" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="I41" s="7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="J41" s="7" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="K41" s="7" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>TRUST FAMILY CARE CENTER, PLLC</t>
+          <t>Marshall Family Chiropractic</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>1 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
@@ -24645,81 +24653,81 @@
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>K-A26</t>
+          <t>K-A03</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Chiropractic</t>
         </is>
       </c>
       <c r="G42" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="I42" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J42" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K42" s="7" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>WESTERN WAYNE PHYSICIANS, PLC</t>
+          <t>Imlay City Family Practice</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>1 visit-day(s) since Mar 3 — re-qualify</t>
+          <t>2 visit-day(s) since Mar 3 — re-qualify</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Jasmine</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>J-A10</t>
+          <t>K-A01</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G43" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>2026-03-27</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="I43" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J43" s="7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>Michigan primary care center/urgent care</t>
+          <t>Holistic Chiropractic</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
@@ -24729,22 +24737,22 @@
       </c>
       <c r="C44" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>Jasmine</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>J-A07</t>
+          <t>C-A14</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Chiropractic</t>
         </is>
       </c>
       <c r="G44" s="7" t="n">
@@ -24752,7 +24760,7 @@
       </c>
       <c r="H44" s="7" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-10-01</t>
         </is>
       </c>
       <c r="I44" s="7" t="n">
@@ -24766,7 +24774,7 @@
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>Burhani Medical Center - use this one</t>
+          <t>BINING AND DAS, MEDICAL GROUP</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -24781,12 +24789,12 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>K-A14</t>
+          <t>C-A15</t>
         </is>
       </c>
       <c r="F45" s="7" t="inlineStr">
@@ -24799,21 +24807,21 @@
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-10-08</t>
         </is>
       </c>
       <c r="I45" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J45" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K45" s="7" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>METROPOLITAN MEDICAL CENTER, PLLC</t>
+          <t>M-15 Family Medical Center</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
@@ -24828,12 +24836,12 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>K-A26</t>
+          <t>C-A02</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
@@ -24846,21 +24854,21 @@
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="I46" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J46" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K46" s="7" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>Macomb Neurology Associates</t>
+          <t>McLaren Oakland Internal Medicine - Clarkston</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -24875,17 +24883,17 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>K-A19</t>
+          <t>C-A02</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Neurology</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G47" s="7" t="n">
@@ -24893,7 +24901,7 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="I47" s="7" t="n">
@@ -24907,7 +24915,7 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>ALAN L FELDMAN, DO, PC</t>
+          <t>Eastlake Cardiovascular</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
@@ -24917,22 +24925,22 @@
       </c>
       <c r="C48" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>Kristen</t>
+          <t>Coty</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>K-A09</t>
+          <t>C-A04</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="G48" s="7" t="n">
@@ -24940,21 +24948,21 @@
       </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="I48" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J48" s="7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K48" s="7" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>Oakland Medical Center</t>
+          <t>TRUST FAMILY CARE CENTER, PLLC</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
@@ -24974,7 +24982,7 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>K-A10</t>
+          <t>K-A26</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
@@ -24987,21 +24995,21 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="I49" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J49" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K49" s="7" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>Trinity IHA Primary &amp; Urgent Care - South Lyon</t>
+          <t>Burhani Medical Center - use this one</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
@@ -25021,7 +25029,7 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>K-A27</t>
+          <t>K-A14</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
@@ -25034,21 +25042,21 @@
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="I50" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J50" s="7" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="K50" s="7" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>One Health</t>
+          <t>METROPOLITAN MEDICAL CENTER, PLLC</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -25058,7 +25066,7 @@
       </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
@@ -25068,7 +25076,7 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>K-A27</t>
+          <t>K-A26</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
@@ -25081,21 +25089,21 @@
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>2026-03-04</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="I51" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J51" s="7" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K51" s="7" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>Priority Medical Center</t>
+          <t>ALAN L FELDMAN, DO, PC</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
@@ -25105,7 +25113,7 @@
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
@@ -25115,7 +25123,7 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>K-A23</t>
+          <t>K-A09</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
@@ -25128,21 +25136,21 @@
       </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="I52" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="J52" s="7" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="K52" s="7" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>Oak Street Health - Pontiac</t>
+          <t>Trinity IHA Primary &amp; Urgent Care - South Lyon</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -25152,7 +25160,7 @@
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -25162,7 +25170,7 @@
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>K-A07</t>
+          <t>K-A27</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
@@ -25175,41 +25183,41 @@
       </c>
       <c r="H53" s="7" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-03-04</t>
         </is>
       </c>
       <c r="I53" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J53" s="7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K53" s="7" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>Western Wayne Family Health Services</t>
+          <t>One Health</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>not visited since Mar 3 — schedule or drop a tier</t>
+          <t>1 visit-day(s) since Mar 3 — re-qualify</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>C-A15</t>
+          <t>K-A27</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
@@ -25218,41 +25226,45 @@
         </is>
       </c>
       <c r="G54" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H54" s="7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>2026-03-04</t>
+        </is>
+      </c>
       <c r="I54" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J54" s="7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K54" s="7" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>WATERFORD PRIMARY HEALTH SERVICES</t>
+          <t>Priority Medical Center</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>not visited since Mar 3 — schedule or drop a tier</t>
+          <t>1 visit-day(s) since Mar 3 — re-qualify</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>C-A02</t>
+          <t>K-A23</t>
         </is>
       </c>
       <c r="F55" s="7" t="inlineStr">
@@ -25261,41 +25273,45 @@
         </is>
       </c>
       <c r="G55" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H55" s="7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-19</t>
+        </is>
+      </c>
       <c r="I55" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J55" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K55" s="7" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>Suzanne Romadan MD</t>
+          <t>Oak Street Health - Pontiac</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>not visited since Mar 3 — schedule or drop a tier</t>
+          <t>1 visit-day(s) since Mar 3 — re-qualify</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>Tier 1</t>
+          <t>Tier 2</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>Coty</t>
+          <t>Kristen</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>C-A04</t>
+          <t>K-A07</t>
         </is>
       </c>
       <c r="F56" s="7" t="inlineStr">
@@ -25304,21 +25320,25 @@
         </is>
       </c>
       <c r="G56" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H56" s="7" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
       <c r="I56" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J56" s="7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="K56" s="7" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>Holistic Chiropractic</t>
+          <t>Western Wayne Family Health Services</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -25338,12 +25358,12 @@
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>C-A14</t>
+          <t>C-A15</t>
         </is>
       </c>
       <c r="F57" s="7" t="inlineStr">
         <is>
-          <t>Chiropractic</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G57" s="7" t="n">
@@ -25351,17 +25371,17 @@
       </c>
       <c r="H57" s="7" t="inlineStr"/>
       <c r="I57" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J57" s="7" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K57" s="7" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>BINING AND DAS, MEDICAL GROUP</t>
+          <t>WATERFORD PRIMARY HEALTH SERVICES</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -25381,7 +25401,7 @@
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>C-A15</t>
+          <t>C-A02</t>
         </is>
       </c>
       <c r="F58" s="7" t="inlineStr">
@@ -25404,7 +25424,7 @@
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>Kidz Care Clinic</t>
+          <t>Suzanne Romadan MD</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
@@ -25424,12 +25444,12 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>C-A01</t>
+          <t>C-A04</t>
         </is>
       </c>
       <c r="F59" s="7" t="inlineStr">
         <is>
-          <t>Pediatrics</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G59" s="7" t="n">
@@ -25437,17 +25457,17 @@
       </c>
       <c r="H59" s="7" t="inlineStr"/>
       <c r="I59" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J59" s="7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K59" s="7" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>Tedd March</t>
+          <t>Kidz Care Clinic</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
@@ -25467,12 +25487,12 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>C-A16</t>
+          <t>C-A01</t>
         </is>
       </c>
       <c r="F60" s="7" t="inlineStr">
         <is>
-          <t>PCP</t>
+          <t>Pediatrics</t>
         </is>
       </c>
       <c r="G60" s="7" t="n">
@@ -25490,7 +25510,7 @@
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>Eastlake Cardiovascular</t>
+          <t>Tedd March</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -25500,7 +25520,7 @@
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>Tier 2</t>
+          <t>Tier 1</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -25510,12 +25530,12 @@
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>C-A04</t>
+          <t>C-A16</t>
         </is>
       </c>
       <c r="F61" s="7" t="inlineStr">
         <is>
-          <t>Other</t>
+          <t>PCP</t>
         </is>
       </c>
       <c r="G61" s="7" t="n">
@@ -25523,10 +25543,10 @@
       </c>
       <c r="H61" s="7" t="inlineStr"/>
       <c r="I61" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J61" s="7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K61" s="7" t="inlineStr"/>
     </row>
@@ -30914,7 +30934,7 @@
         <v>5</v>
       </c>
       <c r="I106" s="7" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J106" s="8" t="n">
         <v>0.426</v>
@@ -30964,7 +30984,7 @@
         <v>1</v>
       </c>
       <c r="I107" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J107" s="8" t="n">
         <v>0.426</v>
@@ -31930,7 +31950,7 @@
         <v>2</v>
       </c>
       <c r="I126" s="7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J126" s="8" t="n">
         <v>0.286</v>
@@ -32706,7 +32726,7 @@
         <v>5</v>
       </c>
       <c r="I142" s="7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J142" s="8" t="n">
         <v>0.267</v>
@@ -32906,7 +32926,7 @@
         <v>2</v>
       </c>
       <c r="I146" s="7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J146" s="8" t="n">
         <v>0.267</v>
@@ -33928,7 +33948,7 @@
         <v>1</v>
       </c>
       <c r="I167" s="7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J167" s="8" t="n">
         <v>0.18</v>
@@ -34274,7 +34294,7 @@
         <v>1</v>
       </c>
       <c r="I174" s="7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J174" s="8" t="n">
         <v>0.18</v>

</xml_diff>